<commit_message>
Remove stripped cylinder-deposit pairs disclosure section
Removed section 2.2 (Stripped cylinder-deposit pairs) from both the .md
and .xlsx versions per request. The main transaction table and Movement
Breakdown are unaffected -- the 5 pairs were already excluded from those,
this only drops the separate audit-trail table listing them.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SaszCD2rHeEEGbAwkQwbeZ
</commit_message>
<xml_diff>
--- a/analysis/debtors/WES004/reports/WES004_Statement_Last3Months_2026-09-16.xlsx
+++ b/analysis/debtors/WES004/reports/WES004_Statement_Last3Months_2026-09-16.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -605,7 +605,7 @@
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>Cylinder-deposit invoice/credit-note pairs that net to zero have been stripped from this view per business_rules.md Rule 11 -- zero impact on the closing balance. See the Stripped Cylinder-Deposit Pairs table below.</t>
+          <t>Cylinder-deposit invoice/credit-note pairs that net to zero have been stripped from this view per business_rules.md Rule 11 -- zero impact on the closing balance.</t>
         </is>
       </c>
     </row>
@@ -1018,251 +1018,76 @@
         <v/>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>Stripped Cylinder-Deposit Pairs (net R0.00, not shown above)</t>
-        </is>
-      </c>
-    </row>
     <row r="35">
-      <c r="A35" s="12" t="inlineStr">
-        <is>
-          <t>Invoice</t>
-        </is>
-      </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>Inv Date</t>
-        </is>
-      </c>
-      <c r="C35" s="12" t="inlineStr">
-        <is>
-          <t>Inv Amount</t>
-        </is>
-      </c>
-      <c r="D35" s="12" t="inlineStr">
-        <is>
-          <t>Crd Note</t>
-        </is>
-      </c>
-      <c r="E35" s="12" t="inlineStr">
-        <is>
-          <t>CN Date</t>
-        </is>
-      </c>
-      <c r="F35" s="12" t="inlineStr">
-        <is>
-          <t>CN Amount</t>
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Reconciliation Sign-off</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="14" t="inlineStr">
-        <is>
-          <t>00051545 (DN#22540=EMPTY)</t>
-        </is>
-      </c>
-      <c r="B36" s="13" t="n">
-        <v>46205</v>
-      </c>
-      <c r="C36" s="15" t="n">
-        <v>2415</v>
-      </c>
-      <c r="D36" s="14" t="inlineStr">
-        <is>
-          <t>00015167</t>
-        </is>
-      </c>
-      <c r="E36" s="13" t="n">
-        <v>46206</v>
-      </c>
-      <c r="F36" s="15" t="n">
-        <v>-2415</v>
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B36" s="17" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>00051859 (DN#22577=EMPTY=)</t>
-        </is>
-      </c>
-      <c r="B37" s="13" t="n">
-        <v>46218</v>
-      </c>
-      <c r="C37" s="15" t="n">
-        <v>2415</v>
-      </c>
-      <c r="D37" s="14" t="inlineStr">
-        <is>
-          <t>00015266</t>
-        </is>
-      </c>
-      <c r="E37" s="13" t="n">
-        <v>46218</v>
-      </c>
-      <c r="F37" s="15" t="n">
-        <v>-2415</v>
+          <t>Combined closing balance (ledger running total)</t>
+        </is>
+      </c>
+      <c r="B37" s="16">
+        <f>B9</f>
+        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>00052200 (DN#23925:EMPTY)</t>
-        </is>
-      </c>
-      <c r="B38" s="13" t="n">
-        <v>46233</v>
-      </c>
-      <c r="C38" s="15" t="n">
-        <v>2415</v>
-      </c>
-      <c r="D38" s="14" t="inlineStr">
-        <is>
-          <t>00015359</t>
-        </is>
-      </c>
-      <c r="E38" s="13" t="n">
-        <v>46234</v>
-      </c>
-      <c r="F38" s="15" t="n">
-        <v>-2415</v>
+          <t>Combined ERP stated balance (WES002 R7,443.73 + WES004 R22,254.14)</t>
+        </is>
+      </c>
+      <c r="B38" s="15" t="n">
+        <v>29697.87</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="14" t="inlineStr">
-        <is>
-          <t>00052668 (DN#22885-EMPTY)</t>
-        </is>
-      </c>
-      <c r="B39" s="13" t="n">
-        <v>46253</v>
-      </c>
-      <c r="C39" s="15" t="n">
-        <v>1207.5</v>
-      </c>
-      <c r="D39" s="14" t="inlineStr">
-        <is>
-          <t>00015502</t>
-        </is>
-      </c>
-      <c r="E39" s="13" t="n">
-        <v>46253</v>
-      </c>
-      <c r="F39" s="15" t="n">
-        <v>-1207.5</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="14" t="inlineStr">
-        <is>
-          <t>00052882 (DN#23991-EMPTY)</t>
-        </is>
-      </c>
-      <c r="B40" s="13" t="n">
-        <v>46265</v>
-      </c>
-      <c r="C40" s="15" t="n">
-        <v>2415</v>
-      </c>
-      <c r="D40" s="14" t="inlineStr">
-        <is>
-          <t>00015577</t>
-        </is>
-      </c>
-      <c r="E40" s="13" t="n">
-        <v>46265</v>
-      </c>
-      <c r="F40" s="15" t="n">
-        <v>-2415</v>
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>Variance</t>
+        </is>
+      </c>
+      <c r="B39" s="10">
+        <f>B37-B38</f>
+        <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="9" t="inlineStr">
-        <is>
-          <t>Net (proof of zero impact)</t>
-        </is>
-      </c>
-      <c r="B41" s="19" t="n"/>
-      <c r="C41" s="19" t="n"/>
-      <c r="D41" s="19" t="n"/>
-      <c r="E41" s="19" t="n"/>
-      <c r="F41" s="10">
-        <f>SUM(C36:C40)+SUM(F36:F40)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>Reconciliation Sign-off</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="17" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="B44" s="17" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="14" t="inlineStr">
-        <is>
-          <t>Combined closing balance (ledger running total)</t>
-        </is>
-      </c>
-      <c r="B45" s="16">
-        <f>B9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="14" t="inlineStr">
-        <is>
-          <t>Combined ERP stated balance (WES002 R7,443.73 + WES004 R22,254.14)</t>
-        </is>
-      </c>
-      <c r="B46" s="15" t="n">
-        <v>29697.87</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="9" t="inlineStr">
-        <is>
-          <t>Variance</t>
-        </is>
-      </c>
-      <c r="B47" s="10">
-        <f>B45-B46</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="11" t="inlineStr">
+      <c r="A41" s="11" t="inlineStr">
         <is>
           <t>Source: WES004_WES002_COMBINED16092026.TXT, built from WES002CURRENT16092026.TXT and WES004CURRENT16092026.TXT ERP account-enquiry exports. Blue cells are figures taken directly from the ERP source; black cells are formulas. Combined collectable balance confirmed by operator 2026-09-16 (see project.json).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="10">
+    <mergeCell ref="A41:F41"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A49:F49"/>
     <mergeCell ref="A13:F13"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A27:F27"/>
-    <mergeCell ref="A34:F34"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A35:F35"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A43:F43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>